<commit_message>
feat: add table_v_sheets to run_meta.json and implement stars matrix generation for Table V correlation; update Excel output structure to include display_stars sheet
</commit_message>
<xml_diff>
--- a/outputs/05_benchmark_signals/tables_v_viii/cn/table_v_correlation.xlsx
+++ b/outputs/05_benchmark_signals/tables_v_viii/cn/table_v_correlation.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="display" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="raw" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="display_stars" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="raw" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1043,6 +1044,635 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:L10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>MOM</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>STR</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>WSTR</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>TREND</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Beta</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Volat.</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>52WH</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Dollar Volume</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Zero Trade</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Size</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Illiq.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>I5/R5</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>-0.01</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>0.13***</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>0.21***</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>-0.03</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>0.11***</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>0.06***</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>-0.07***</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>0.08***</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>-0.29***</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>0.03**</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>-0.05***</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>I5/R20</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>-0.01</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>0.14***</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>0.24***</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>0.06***</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>0.05***</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>-0.09***</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>-0.01</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>-0.13***</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>-0.04***</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>I5/R60</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>-0.03**</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>-0.00</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>-0.00</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>-0.02**</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>-0.02**</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>-0.03***</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>-0.03***</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>0.02**</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>I20/R5</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>-0.01</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>0.09***</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>0.13***</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>0.10***</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>0.05</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>-0.06***</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>0.05*</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>-0.27***</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>-0.03***</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>I20/R20</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>-0.00</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>0.13***</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>0.12***</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>0.04***</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>0.02</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>-0.07***</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>-0.04***</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>-0.04***</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>-0.04***</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>I20/R60</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>0.02</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>-0.03***</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>0.03***</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>-0.04**</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>-0.01</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>0.02</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>0.02</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>-0.01</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>0.03*</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>-0.02</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>I60/R5</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>-0.01</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>0.07***</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>0.10***</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>0.09***</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>0.03</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>-0.03</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>0.03*</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>-0.25***</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>-0.02</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>0.02</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>I60/R20</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>-0.00</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>0.09***</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>0.06***</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>0.02</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>-0.03***</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>-0.04***</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>-0.06***</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>-0.03**</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>-0.03*</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>0.02</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>I60/R60</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>0.03</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>-0.01</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>0.02**</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>-0.05***</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>-0.02</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>0.06***</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>0.02</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>0.02</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>0.03</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>-0.01</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>-0.02</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:W10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>